<commit_message>
Literature matrix: builder script, verified data file, four related efficiency papers (18 total)
</commit_message>
<xml_diff>
--- a/deliverables/literature_matrix.xlsx
+++ b/deliverables/literature_matrix.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="355" uniqueCount="309">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="369">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -658,6 +658,180 @@
     <t xml:space="preserve">https://arxiv.org/abs/2506.07339</t>
   </si>
   <si>
+    <t xml:space="preserve">RealtimeVLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running VLAs at Real-time Speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yunchao Ma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arXiv (2510.26742)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pi0-level VLA: PaliGemma backbone (SigLIP ~400M + Gemma 2.6B, ~3B) + ~300M action expert.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flow matching, 10 action-expert denoising steps (pi0 recipe).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inference-only systems optimisation: CUDA graphs to remove CPU launch overhead (~2x), folding RMSNorm affine and the action-time embedding into adjacent linear layers, fused QKV/RoPE, fused gated linear layers and scalar ops, Triton GEMM tile tuning, dropping the last LLM layer (17 of 18); plus a streaming inference framework.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency (CPU launch overhead, kernel fusion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTX 4090, bf16, 10 steps (Table 1): 2 views 106.5 ms (naive torch) / 53.7 ms (openpi JAX) -&gt; 27.3 ms; 1 view 20.0 ms; 3 views 36.8 ms; 30 Hz frame rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real-world falling-pen catching: 10/10 consecutive successes (policy trained with openpi on 600 episodes). No standard benchmark reported.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model weights fixed; a single consumer GPU with native bf16; per-shape kernel tuning for one model and input size.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large engineering effort (hand-written/fused kernels) tied to one architecture and GPU; dropping a layer changes the model; no closed-loop success comparison against the unoptimised policy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(reviewer inference) Whether each fused/approximated step leaves closed-loop success unchanged on a standard benchmark; portability to GPUs without bf16 tensor cores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes (speed-ups); the task policy itself was trained</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2510.26742</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Islam-ONNX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When Faster VLA Deployment Changes Closed-Loop Behavior: Task Success-Latency Analysis of SmolVLA Across PyTorch and ONNX Variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rafiqul Islam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arXiv (2609.14146)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same checkpoint as this study: HuggingFaceVLA/smolvla_libero, LeRobot 0.6.1 (MuJoCo 3.3.2).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flow matching, 10 flow steps (released configuration).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runtime change: PyTorch+AMP vs ONNX Runtime (CUDA EP) with 'requested' FP16/INT8 exports; static language width 16/24/32 tokens.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency (runtime/export), closed-loop side effects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTX 2060 6 GB, batch 1: PyTorch+AMP p50 903 ms / p99 1181 ms; ONNX p50 537.5-549.2 ms (p99 532-601 ms) - about 2x lower latency.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIBERO Spatial / Object, 100 episodes each: PyTorch+AMP 70.0 / 88.0; ONNX width 16 41.0 / 89.0; width 24 75.0 / 90.0; width 32 71.0 / 87.0. Paired 300 episodes, Spatial: 56.7 vs 33.0 (McNemar p = 2.2e-9).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One GPU, one checkpoint, one seed; the exported graph has a static language width (width 16 truncates 5 of 10 Spatial instructions).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faster runtime but a silent behaviour change: truncated instructions cut Spatial success by ~29 pp; the 'INT8' artifact is a byte-identical FP32 graph, i.e. not real INT8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors: factors other than width (graph conversion, AMP vs FP32, kernels, true INT8, TensorRT) not isolated; no equivalence test ('a non-significant two-proportion test is not an equivalence result').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2609.14146</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fewer Steps, Better Actions: Rethinking Flow-Matching Inference for VLA Policies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zhipeng Tang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arXiv (2609.21216)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frozen pi0.5 (fine-tuned) and frozen official SmolVLA; corrector parameter count UNVERIFIED (not reported).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flow matching with few Euler steps + a learned endpoint correction (lightweight Transformer reading the candidate action, the source noise and the shared prefix cache).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spend part of the integration budget on a learned residual corrector instead of more flow steps.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency (fewer flow steps + learned correction)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pi0.5-FT on A100: 10 steps 233.0 ms -&gt; Coda 2 steps 109.9 ms (2.12x); SmolVLA: 233.5 -&gt; 118.1 ms (1.98x).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RoboTwin Easy (50 tasks), pi0.5-FT naive steps 1/2/3/5/10: 59.76/67.40/71.28/71.64/71.52%; Coda 2 steps 71.88%. SmolVLA (10 tasks) naive 1/2/5/10: 35.0/60.8/60.8/64.4%; Coda 2 steps 69.4%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demonstrations available to train the corrector (SmolVLA: 18,716 steps, batch 256); base policy frozen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires training and a second network; naive step reduction alone is nearly free for pi0.5 down to 3 steps but collapses at 1 step (and for SmolVLA at 1 step).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(reviewer inference) Results are on RoboTwin; whether the same step curve holds on LIBERO and for per-step re-planning.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no (corrector only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2609.21216</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vla.cpp</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vla.cpp: A Unified Inference Runtime for Vision-Language-Action Models</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Khanh D. Nguyen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arXiv (2606.08094)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C++ runtime for eleven VLA models (list UNVERIFIED from the abstract); SmolVLA and BitVLA discussed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Architecture-specific heads; iterative policies reuse observation-dependent computation across solver steps.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runtime without PyTorch: shared loading/execution/serving; ternary tensor-core kernel for BitVLA.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency, memory, edge deployment (runtime)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BitVLA client inference 4.0-4.6x faster than a CUDA-core baseline on RTX 3060 and AGX Orin.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIBERO-Object: BitVLA 200/200 episodes on an 8 GB Jetson Orin Nano; a SmolVLA case study links positional-index precision to gripper commands and task success.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Re-implementation of each model in C++ matches the reference behaviour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineering cost per architecture; numerical details (e.g. positional-index precision) can change closed-loop behaviour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(reviewer inference) Absolute latencies and SmolVLA success rates not given in the abstract.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2606.08094</t>
+  </si>
+  <si>
     <t xml:space="preserve">Model</t>
   </si>
   <si>
@@ -790,7 +964,7 @@
     <t xml:space="preserve">n=50; this checkpoint executes 1 action per re-plan</t>
   </si>
   <si>
-    <t xml:space="preserve">This study, Tesla T4: 814 ms per re-plan (bf16, 10 steps)</t>
+    <t xml:space="preserve">This study, Tesla T4: 789 ms per re-plan (bf16, 10 steps)</t>
   </si>
   <si>
     <t xml:space="preserve">arxiv.org/abs/2506.01844; LeRobot v0.6.1</t>
@@ -835,13 +1009,13 @@
     <t xml:space="preserve">2. Path: the DDPM forward process follows a variance-preserving schedule (curved trajectories under the probability-flow ODE); the linear flow path has constant velocity per sample, so coarse Euler steps stay close (this study: 3 steps deviate 0.32 vs a 1.37 sampling spread, LIBERO-Object).</t>
   </si>
   <si>
-    <t xml:space="preserve">3. Sampling: DDPM needs many steps (DDIM ~10); flow models use ~10 Euler steps by default and degrade gracefully when fewer are used.</t>
+    <t xml:space="preserve">3. Sampling: DDPM needs many steps (DDIM ~10); flow models use ~10 Euler steps by default and degrade gracefully when fewer are used, down to a model-dependent limit (Coda: pi0.5 holds at 3 steps, drops at 1; SmolVLA drops at 1).</t>
   </si>
   <si>
     <t xml:space="preserve">4. Cost per step: in all four VLA-style models a step re-runs only a small head on a cached VLM output, so per-step cost is set by the head size and by kernel-launch overhead at batch 1.</t>
   </si>
   <si>
-    <t xml:space="preserve">SmolVLA (HuggingFaceVLA/smolvla_libero) on LIBERO-Spatial, Tesla T4 - latency of one re-plan (median, CUDA events)</t>
+    <t xml:space="preserve">SmolVLA (HuggingFaceVLA/smolvla_libero) on LIBERO-Spatial, Tesla T4 - latency of one re-plan (median, CUDA events, results/t4/profile/graph_t4.json)</t>
   </si>
   <si>
     <t xml:space="preserve">Configuration</t>
@@ -868,9 +1042,6 @@
     <t xml:space="preserve">bf16</t>
   </si>
   <si>
-    <t xml:space="preserve">results/t4/profile/graph_t4.json</t>
-  </si>
-  <si>
     <t xml:space="preserve">Fewer steps</t>
   </si>
   <si>
@@ -886,7 +1057,7 @@
     <t xml:space="preserve">fp16, 3 steps</t>
   </si>
   <si>
-    <t xml:space="preserve">fp16, 3 steps + graph (proposed)</t>
+    <t xml:space="preserve">fp16, 3 steps + graph</t>
   </si>
   <si>
     <t xml:space="preserve">fp16, 2 steps + graph</t>
@@ -895,10 +1066,13 @@
     <t xml:space="preserve">fp16, 1 step + graph</t>
   </si>
   <si>
-    <t xml:space="preserve">Blue numbers are measured inputs (bench_graph, 60 calls per configuration after warm-up, interleaved rounds); speed-ups are formulas against the released configuration.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Configuration (paired, same 200 episodes, common random numbers)</t>
+    <t xml:space="preserve">Blue numbers are measured inputs (60 calls per configuration after warm-up, interleaved rounds); speed-ups are formulas against the released configuration.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configuration (paired, same episodes, common random numbers)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n</t>
   </si>
   <si>
     <t xml:space="preserve">Success rate</t>
@@ -937,7 +1111,7 @@
     <t xml:space="preserve">Open loop, 10 actions per re-plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: results/t4/summary.json (Newcombe paired CI; exact McNemar). Non-inferiority margin: -5 pp.</t>
+    <t xml:space="preserve">Source: results/t4/summary.json (Newcombe paired CI; exact McNemar, unadjusted). Non-inferiority margin: -5 pp.</t>
   </si>
   <si>
     <t xml:space="preserve">How this matrix was built: every entry was read from the paper's own arXiv abstract, HTML or PDF (column 'Source'). 'UNVERIFIED' marks values not found in the text that was read; '(reviewer inference)' marks open questions that are our reading, not the authors' statement.</t>
@@ -947,6 +1121,12 @@
   </si>
   <si>
     <t xml:space="preserve">A2C2 trains its own SmolVLA from scratch on LIBERO; its execution-horizon results (e=5: 0.83 &gt; e=1: 0.77) are not for the checkpoint used in this study, for which executing 5 actions per re-plan lowers SR by 12.5 pp.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Islam (2026) uses the same checkpoint and LeRobot version on a Turing GPU (RTX 2060): its PyTorch+AMP Spatial success (70.0%, 100 episodes) is in the range of this study's baseline (77.0%, 200 episodes); its ONNX speed-up came with a behaviour change (truncated instructions), which motivates checking closed-loop equivalence for every efficiency change.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coda (2026) and Realtime-VLA (2025) already apply fewer flow steps and CUDA graphs, respectively; this study does not claim these levers as new.</t>
   </si>
   <si>
     <t xml:space="preserve">Venues for pi0, OpenVLA and OpenVLA-OFT are not stated on the arXiv pages read and are left as arXiv.</t>
@@ -956,13 +1136,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.00\x"/>
-    <numFmt numFmtId="167" formatCode="0.0%"/>
-    <numFmt numFmtId="168" formatCode="\+0.0;\-0.0;0.0"/>
-    <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0"/>
+    <numFmt numFmtId="168" formatCode="0.0%"/>
+    <numFmt numFmtId="169" formatCode="\+0.0;\-0.0;0.0"/>
+    <numFmt numFmtId="170" formatCode="0.000"/>
   </numFmts>
   <fonts count="11">
     <font>
@@ -1106,7 +1287,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1172,6 +1353,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="169" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1435,7 +1620,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P15"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -2201,6 +2386,206 @@
       </c>
       <c r="P15" s="5" t="s">
         <v>210</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2" t="s">
+        <v>211</v>
+      </c>
+      <c r="B16" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>213</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>2025</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>215</v>
+      </c>
+      <c r="G16" s="3" t="s">
+        <v>216</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>217</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>218</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>219</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="L16" s="3" t="s">
+        <v>221</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>222</v>
+      </c>
+      <c r="N16" s="3" t="s">
+        <v>223</v>
+      </c>
+      <c r="O16" s="3" t="s">
+        <v>224</v>
+      </c>
+      <c r="P16" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="B17" s="5" t="s">
+        <v>227</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E17" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="F17" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="G17" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="H17" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="I17" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="M17" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="N17" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="O17" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="P17" s="5" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
+        <v>240</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E18" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="G18" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="H18" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="I18" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="J18" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="K18" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="L18" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="M18" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="N18" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="O18" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="P18" s="3" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>255</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>258</v>
+      </c>
+      <c r="F19" s="5" t="s">
+        <v>259</v>
+      </c>
+      <c r="G19" s="5" t="s">
+        <v>260</v>
+      </c>
+      <c r="H19" s="5" t="s">
+        <v>261</v>
+      </c>
+      <c r="I19" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="J19" s="5" t="s">
+        <v>263</v>
+      </c>
+      <c r="K19" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="L19" s="5" t="s">
+        <v>265</v>
+      </c>
+      <c r="M19" s="5" t="s">
+        <v>266</v>
+      </c>
+      <c r="N19" s="5" t="s">
+        <v>267</v>
+      </c>
+      <c r="O19" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="P19" s="5" t="s">
+        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -2235,66 +2620,66 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>211</v>
+        <v>269</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>212</v>
+        <v>270</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>213</v>
+        <v>271</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>214</v>
+        <v>272</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>215</v>
+        <v>273</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>216</v>
+        <v>274</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>217</v>
+        <v>275</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>218</v>
+        <v>276</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>219</v>
+        <v>277</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>220</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>221</v>
+        <v>279</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>222</v>
+        <v>280</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>223</v>
+        <v>281</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>224</v>
+        <v>282</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>225</v>
+        <v>283</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>226</v>
+        <v>284</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>227</v>
+        <v>285</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>228</v>
+        <v>286</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>229</v>
+        <v>287</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>230</v>
+        <v>288</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2302,31 +2687,31 @@
         <v>170</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>231</v>
+        <v>289</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>223</v>
+        <v>281</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>232</v>
+        <v>290</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>233</v>
+        <v>291</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>234</v>
+        <v>292</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>235</v>
+        <v>293</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>236</v>
+        <v>294</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>237</v>
+        <v>295</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>238</v>
+        <v>296</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2334,105 +2719,105 @@
         <v>31</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>239</v>
+        <v>297</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>240</v>
+        <v>298</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>241</v>
+        <v>299</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>242</v>
+        <v>300</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>243</v>
+        <v>301</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>244</v>
+        <v>302</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>245</v>
+        <v>303</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>246</v>
+        <v>304</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>247</v>
+        <v>305</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>248</v>
+        <v>306</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>239</v>
+        <v>297</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>249</v>
+        <v>307</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>250</v>
+        <v>308</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>251</v>
+        <v>309</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>252</v>
+        <v>310</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>253</v>
+        <v>311</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>254</v>
+        <v>312</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>255</v>
+        <v>313</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>256</v>
+        <v>314</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>257</v>
+        <v>315</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>258</v>
+        <v>316</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>259</v>
+        <v>317</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>260</v>
+        <v>318</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>261</v>
+        <v>319</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>262</v>
+        <v>320</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>263</v>
+        <v>321</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>264</v>
+        <v>322</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>265</v>
+        <v>323</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>266</v>
+        <v>324</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>268</v>
+        <v>326</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -2444,9 +2829,9 @@
       <c r="I9" s="7"/>
       <c r="J9" s="7"/>
     </row>
-    <row r="10" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>269</v>
+        <v>327</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -2458,9 +2843,9 @@
       <c r="I10" s="7"/>
       <c r="J10" s="7"/>
     </row>
-    <row r="11" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>270</v>
+        <v>328</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -2472,9 +2857,9 @@
       <c r="I11" s="7"/>
       <c r="J11" s="7"/>
     </row>
-    <row r="12" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>271</v>
+        <v>329</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -2508,50 +2893,48 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>272</v>
+        <v>330</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>273</v>
+        <v>331</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>274</v>
+        <v>332</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>275</v>
+        <v>333</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>276</v>
+        <v>334</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>277</v>
+        <v>335</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>278</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>220</v>
+        <v>336</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>279</v>
+        <v>337</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>280</v>
+        <v>338</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>10</v>
@@ -2566,16 +2949,13 @@
         <f aca="false">$E$4/E4</f>
         <v>1</v>
       </c>
-      <c r="G4" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>282</v>
+        <v>339</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>280</v>
+        <v>338</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>3</v>
@@ -2590,16 +2970,13 @@
         <f aca="false">$E$4/E5</f>
         <v>1.82389646406286</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>283</v>
+        <v>340</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>280</v>
+        <v>338</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>10</v>
@@ -2614,16 +2991,13 @@
         <f aca="false">$E$4/E6</f>
         <v>1.37972027972028</v>
       </c>
-      <c r="G6" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>284</v>
+        <v>341</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>284</v>
+        <v>341</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>10</v>
@@ -2638,16 +3012,13 @@
         <f aca="false">$E$4/E7</f>
         <v>1.28096088297354</v>
       </c>
-      <c r="G7" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>285</v>
+        <v>342</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>284</v>
+        <v>341</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>10</v>
@@ -2662,16 +3033,13 @@
         <f aca="false">$E$4/E8</f>
         <v>4.43370786516854</v>
       </c>
-      <c r="G8" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>286</v>
+        <v>343</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>284</v>
+        <v>341</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>3</v>
@@ -2686,16 +3054,13 @@
         <f aca="false">$E$4/E9</f>
         <v>3.21859706362153</v>
       </c>
-      <c r="G9" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>287</v>
+        <v>344</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>284</v>
+        <v>341</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>3</v>
@@ -2710,16 +3075,13 @@
         <f aca="false">$E$4/E10</f>
         <v>7.05272564789991</v>
       </c>
-      <c r="G10" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>288</v>
+        <v>345</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>284</v>
+        <v>341</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>2</v>
@@ -2734,16 +3096,13 @@
         <f aca="false">$E$4/E11</f>
         <v>7.64728682170543</v>
       </c>
-      <c r="G11" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>289</v>
+        <v>346</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>284</v>
+        <v>341</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>1</v>
@@ -2758,196 +3117,217 @@
         <f aca="false">$E$4/E12</f>
         <v>8.45873526259378</v>
       </c>
-      <c r="G12" s="10" t="s">
-        <v>281</v>
-      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>290</v>
+        <v>347</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>291</v>
+        <v>348</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>292</v>
+        <v>349</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>293</v>
+        <v>350</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>294</v>
+        <v>351</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>295</v>
+        <v>352</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>296</v>
+        <v>353</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>297</v>
+        <v>354</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>355</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>298</v>
+        <v>356</v>
       </c>
       <c r="B17" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C17" s="15" t="n">
         <v>0.77</v>
       </c>
-      <c r="C17" s="15" t="n">
+      <c r="D17" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D17" s="15"/>
-      <c r="E17" s="15"/>
+      <c r="E17" s="16"/>
       <c r="F17" s="16"/>
-      <c r="G17" s="17" t="n">
+      <c r="G17" s="17"/>
+      <c r="H17" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>299</v>
+        <v>357</v>
       </c>
       <c r="B18" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C18" s="15" t="n">
         <v>0.79</v>
       </c>
-      <c r="C18" s="15" t="n">
+      <c r="D18" s="16" t="n">
         <v>2</v>
       </c>
-      <c r="D18" s="15" t="n">
+      <c r="E18" s="16" t="n">
         <v>-3.82675992832326</v>
       </c>
-      <c r="E18" s="15" t="n">
+      <c r="F18" s="16" t="n">
         <v>7.83816136488135</v>
       </c>
-      <c r="F18" s="16" t="n">
+      <c r="G18" s="17" t="n">
         <v>0.60759136127308</v>
       </c>
-      <c r="G18" s="17" t="n">
+      <c r="H18" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>286</v>
+        <v>343</v>
       </c>
       <c r="B19" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C19" s="15" t="n">
         <v>0.77</v>
       </c>
-      <c r="C19" s="15" t="n">
+      <c r="D19" s="16" t="n">
         <v>0</v>
       </c>
-      <c r="D19" s="15" t="n">
+      <c r="E19" s="16" t="n">
         <v>-5.83223180674493</v>
       </c>
-      <c r="E19" s="15" t="n">
+      <c r="F19" s="16" t="n">
         <v>5.83223180674493</v>
       </c>
-      <c r="F19" s="16" t="n">
+      <c r="G19" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="G19" s="17" t="n">
+      <c r="H19" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>300</v>
+        <v>358</v>
       </c>
       <c r="B20" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C20" s="15" t="n">
         <v>0.65</v>
       </c>
-      <c r="C20" s="15" t="n">
+      <c r="D20" s="16" t="n">
         <v>-12</v>
       </c>
-      <c r="D20" s="15" t="n">
+      <c r="E20" s="16" t="n">
         <v>-19.1121708723983</v>
       </c>
-      <c r="E20" s="15" t="n">
+      <c r="F20" s="16" t="n">
         <v>-4.7396645919743</v>
       </c>
-      <c r="F20" s="16" t="n">
+      <c r="G20" s="17" t="n">
         <v>0.00184155478849254</v>
       </c>
-      <c r="G20" s="17" t="n">
+      <c r="H20" s="18" t="n">
         <v>100</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>301</v>
+        <v>359</v>
       </c>
       <c r="B21" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C21" s="15" t="n">
         <v>0.645</v>
       </c>
-      <c r="C21" s="15" t="n">
+      <c r="D21" s="16" t="n">
         <v>-12.5</v>
       </c>
-      <c r="D21" s="15" t="n">
+      <c r="E21" s="16" t="n">
         <v>-20.2579444201042</v>
       </c>
-      <c r="E21" s="15" t="n">
+      <c r="F21" s="16" t="n">
         <v>-4.53918860259062</v>
       </c>
-      <c r="F21" s="16" t="n">
+      <c r="G21" s="17" t="n">
         <v>0.00306531766960874</v>
       </c>
-      <c r="G21" s="17" t="n">
+      <c r="H21" s="18" t="n">
         <v>20.1451960754534</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>302</v>
+        <v>360</v>
       </c>
       <c r="B22" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C22" s="15" t="n">
         <v>0.65</v>
       </c>
-      <c r="C22" s="15" t="n">
+      <c r="D22" s="16" t="n">
         <v>-12</v>
       </c>
-      <c r="D22" s="15" t="n">
+      <c r="E22" s="16" t="n">
         <v>-18.7213903156737</v>
       </c>
-      <c r="E22" s="15" t="n">
+      <c r="F22" s="16" t="n">
         <v>-5.15896130609279</v>
       </c>
-      <c r="F22" s="16" t="n">
+      <c r="G22" s="17" t="n">
         <v>0.000936222910851825</v>
       </c>
-      <c r="G22" s="17" t="n">
+      <c r="H22" s="18" t="n">
         <v>21.4708394338702</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>303</v>
+        <v>361</v>
       </c>
       <c r="B23" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C23" s="15" t="n">
         <v>0.675</v>
       </c>
-      <c r="C23" s="15" t="n">
+      <c r="D23" s="16" t="n">
         <v>-9.5</v>
       </c>
-      <c r="D23" s="15" t="n">
+      <c r="E23" s="16" t="n">
         <v>-17.2512236724465</v>
       </c>
-      <c r="E23" s="15" t="n">
+      <c r="F23" s="16" t="n">
         <v>-1.60394995079444</v>
       </c>
-      <c r="F23" s="16" t="n">
+      <c r="G23" s="17" t="n">
         <v>0.0248119745715522</v>
       </c>
-      <c r="G23" s="17" t="n">
+      <c r="H23" s="18" t="n">
         <v>10.1963346712717</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>304</v>
+        <v>362</v>
       </c>
     </row>
   </sheetData>
@@ -2966,30 +3346,40 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="140"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
-        <v>305</v>
+      <c r="A1" s="19" t="s">
+        <v>363</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="18" t="s">
-        <v>306</v>
+      <c r="A2" s="19" t="s">
+        <v>364</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="18" t="s">
-        <v>307</v>
+      <c r="A3" s="19" t="s">
+        <v>365</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="18" t="s">
-        <v>308</v>
+      <c r="A4" s="19" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="19" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="19" t="s">
+        <v>368</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Final S=1 confirmation in report, README results, literature matrix and summary
</commit_message>
<xml_diff>
--- a/deliverables/literature_matrix.xlsx
+++ b/deliverables/literature_matrix.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="369">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="372">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -1111,10 +1111,19 @@
     <t xml:space="preserve">Open loop, 10 actions per re-plan</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: results/t4/summary.json (Newcombe paired CI; exact McNemar, unadjusted). Non-inferiority margin: -5 pp.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">How this matrix was built: every entry was read from the paper's own arXiv abstract, HTML or PDF (column 'Source'). 'UNVERIFIED' marks values not found in the text that was read; '(reviewer inference)' marks open questions that are our reading, not the authors' statement.</t>
+    <t xml:space="preserve">fp16, 2 steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fp16, 1 step</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fp16, 3 steps, one fixed noise per episode (probe)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source: results/t4/summary.json (Newcombe paired CI; exact McNemar, unadjusted). Non-inferiority margin: -5 pp. fp16 1 step pools the exploratory states 0-19 with the confirmation states 20-49; the pre-specified test on states 20-49 alone gives +6.0 pp [+0.6, +11.4], p = 0.04 (results/t4/report_numbers.json).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How this matrix was built: every entry was read from the paper's own arXiv abstract, HTML or PDF (column 'Source'). 'UNVERIFIED' marks values not found in the text that was read; '(reviewer inference)' marks open questions that are the reviewer's reading, not the authors' statement.</t>
   </si>
   <si>
     <t xml:space="preserve">Inconsistencies found in the sources: Diffusion Policy states 10 DDIM inference steps (Sec. 3.4) and 16 (App. A.4); VLA-Cache's 1.7x headline is larger than its per-model tables (OpenVLA 1.63x); TinyVLA text and tables differ (44.5% vs 47.8%); A2C2 Table 1 and Table 7 differ for the same settings and its LIBERO tables contain no RTC column.</t>
@@ -2893,7 +2902,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -3154,10 +3163,10 @@
         <v>356</v>
       </c>
       <c r="B17" s="14" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C17" s="15" t="n">
-        <v>0.77</v>
+        <v>0.754</v>
       </c>
       <c r="D17" s="16" t="n">
         <v>0</v>
@@ -3200,22 +3209,22 @@
         <v>343</v>
       </c>
       <c r="B19" s="14" t="n">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C19" s="15" t="n">
-        <v>0.77</v>
+        <v>0.784</v>
       </c>
       <c r="D19" s="16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E19" s="16" t="n">
-        <v>-5.83223180674493</v>
+        <v>-0.631992837712167</v>
       </c>
       <c r="F19" s="16" t="n">
-        <v>5.83223180674493</v>
+        <v>6.63807721057419</v>
       </c>
       <c r="G19" s="17" t="n">
-        <v>1</v>
+        <v>0.128396402926401</v>
       </c>
       <c r="H19" s="18" t="n">
         <v>100</v>
@@ -3325,9 +3334,87 @@
         <v>10.1963346712717</v>
       </c>
     </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="9" t="s">
+        <v>362</v>
+      </c>
+      <c r="B24" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C24" s="15" t="n">
+        <v>0.775</v>
+      </c>
+      <c r="D24" s="16" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E24" s="16" t="n">
+        <v>-5.72404100060382</v>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>6.72438487868041</v>
+      </c>
+      <c r="G24" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="H24" s="18" t="n">
+        <v>100</v>
+      </c>
+    </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="13" t="s">
-        <v>362</v>
+      <c r="A25" s="9" t="s">
+        <v>363</v>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>500</v>
+      </c>
+      <c r="C25" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D25" s="16" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="E25" s="16" t="n">
+        <v>0.426718068789581</v>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>8.7695987253317</v>
+      </c>
+      <c r="G25" s="17" t="n">
+        <v>0.0380186455827965</v>
+      </c>
+      <c r="H25" s="18" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
+        <v>364</v>
+      </c>
+      <c r="B26" s="14" t="n">
+        <v>200</v>
+      </c>
+      <c r="C26" s="15" t="n">
+        <v>0.235</v>
+      </c>
+      <c r="D26" s="16" t="n">
+        <v>-53.5</v>
+      </c>
+      <c r="E26" s="16" t="n">
+        <v>-60.3219004894075</v>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>-45.3845150827603</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <v>3.450744533327E-028</v>
+      </c>
+      <c r="H26" s="18" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="13" t="s">
+        <v>365</v>
       </c>
     </row>
   </sheetData>
@@ -3354,32 +3441,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Literature matrix: ten core papers with a relevance column; report wording on graph replay and matrix size
</commit_message>
<xml_diff>
--- a/deliverables/literature_matrix.xlsx
+++ b/deliverables/literature_matrix.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="411" uniqueCount="372">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="274">
   <si>
     <t xml:space="preserve">ID</t>
   </si>
@@ -40,6 +40,9 @@
     <t xml:space="preserve">Venue / arXiv</t>
   </si>
   <si>
+    <t xml:space="preserve">Relevance to this study</t>
+  </si>
+  <si>
     <t xml:space="preserve">Model size &amp; backbone</t>
   </si>
   <si>
@@ -85,6 +88,9 @@
     <t xml:space="preserve">arXiv (2506.01844)</t>
   </si>
   <si>
+    <t xml:space="preserve">The model studied: its LIBERO checkpoint is reproduced and optimised here.</t>
+  </si>
+  <si>
     <t xml:space="preserve">0.45B total (Table 5; also 0.24B and 2.25B variants). VLM = SmolVLM-2 (SigLIP vision encoder + SmolLM2 decoder); only first N=L/2 VLM layers used (last L-N skipped); 64 visual tokens per frame (global image, no tiling). Action expert hidden size 0.75×d of VLM (expert param count UNVERIFIED).</t>
   </si>
   <si>
@@ -130,6 +136,9 @@
     <t xml:space="preserve">arXiv (RSS 2025 per external listings; not stated on arXiv page read — UNVERIFIED) (2410.24164)</t>
   </si>
   <si>
+    <t xml:space="preserve">Same design as SmolVLA (VLM prefix + flow-matching action expert, 10 Euler steps on a cached prefix).</t>
+  </si>
+  <si>
     <t xml:space="preserve">3.3B total: PaliGemma 3B VLM + ~300M action expert (width=1024, mlp dim=4096, initialized from scratch)</t>
   </si>
   <si>
@@ -160,46 +169,49 @@
     <t xml:space="preserve">https://arxiv.org/abs/2410.24164</t>
   </si>
   <si>
-    <t xml:space="preserve">OpenVLA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OpenVLA: An Open-Source Vision-Language-Action Model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Moo Jin Kim (co-first with Karl Pertsch, Siddharth Karamcheti)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (CoRL 2024 per external listings; not stated in PDF read — UNVERIFIED) (2406.09246)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7B; Prismatic-7B VLM: fused DINOv2+SigLIP vision encoder (~600M, features concatenated channel-wise), 2-layer MLP projector, Llama 2 7B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">autoregressive tokens: each action dimension discretized into 256 bins (1st–99th quantile), mapped onto the 256 least-used Llama tokens; one action per step (7 tokens), no chunking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parameter-efficient adaptation (LoRA, 1.4% of params) and memory-efficient inference via int8/int4 quantization; baseline efficiency reference for later work</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Memory (quantisation), fine-tuning cost (LoRA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vs RT-2-X (55B): +16.5% absolute task success across 29 tasks with 7× fewer params. LoRA: 1.4% params, matches full FT; 10–15 h on 1 A100 vs full FT 8 A100 × 5–15 h (8× compute reduction). Quantization (Table 2, BridgeData V2): bf16 71.3% / 16.8 GB; int8 58.1% / 10.2 GB; int4 71.9% / 7.0 GB; on A5000 int8 1.2 Hz, int4 3 Hz. ~6 Hz bf16 on RTX 4090 (no compilation/speculative decoding).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">29-task real-robot eval vs RT-2-X (+16.5% abs). LIBERO fine-tuned (S/O/G/L/avg) 84.7/88.4/79.2/53.7/76.5 as reported in the SmolVLA paper's table (not verified in OpenVLA PDF excerpt read).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Single-image observation, no proprioception or history; discretized actions sufficient; 970k OXE demonstrations for pretraining.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Autoregressive per-dimension decoding limits throughput (~6 Hz on RTX 4090); int8 quantization hurt success (58.1%) and was slower (1.2 Hz) than int4 on A5000.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors: need higher inference throughput for high-frequency control (e.g., ALOHA 50 Hz); single-image only; success typically &lt;90%. (reviewer inference) Effect of action chunking/parallel decoding (later answered by OpenVLA-OFT).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2406.09246</t>
+    <t xml:space="preserve">DiffusionPolicy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diffusion Policy: Visuomotor Policy Learning via Action Diffusion</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cheng Chi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSS 2023 (conference version); arXiv PDF read is the extended version (journal not named on the page) (2303.04137)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reference diffusion action head for the diffusion vs flow-matching comparison.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not a VLA (no language model). ResNet-18 vision encoder (~22M, trained end-to-end); CNN-based diffusion net ~22M (45M Transport) or time-series diffusion transformer ~9M (sim) / 80M (Kitchen, real Push-T)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">diffusion (DDPM, epsilon/noise-prediction MSE objective conditioned on observations); sim: 100 denoising iterations for training and inference; real: DDIM with 100 training / 10 inference iterations (Appendix A.4 says 16 — inconsistent); To=2, Tp=16, Ta=8 (receding-horizon control)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Not an efficiency paper; DDIM reduces inference iterations (100 -&gt; 10) and action-sequence prediction with receding horizon amortizes inference over Ta=8 executed actions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">N/A (generative action-head reference)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">'0.1s inference latency on a Nvidia 3080 GPU' (DDIM, 10 inference iterations, real world)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average improvement of 46.9% over prior methods (abstract of version read: 15 tasks from 4 benchmarks; Table 3: 12 tasks, 8 sim + 4 real). Third-party: LIBERO avg 72.4 (scratch) in OpenVLA-OFT/SmolVLA tables; Meta-World avg 10.5 in TinyVLA/SmolVLA tables.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sufficient task-specific demonstrations (behavior cloning); actions executed open-loop for Ta steps between replans; multimodal action distributions benefit from diffusion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors: higher compute and inference latency than simpler methods such as LSTM-GMM; action-sequence prediction may not suffice for high-rate control tasks.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors: inherits behavior-cloning limits (poor with inadequate demos). (reviewer inference) Few-step / consistency distillation for faster sampling; scaling with language conditioning (addressed by later VLAs).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2303.04137</t>
   </si>
   <si>
     <t xml:space="preserve">OpenVLA-OFT</t>
@@ -214,6 +226,9 @@
     <t xml:space="preserve">arXiv (RSS 2025 per external listings; not stated in PDF v2 read — UNVERIFIED) (2502.19645)</t>
   </si>
   <si>
+    <t xml:space="preserve">Reports speed and success together; chunked parallel decoding is the 'execute more per call' idea.</t>
+  </si>
+  <si>
     <t xml:space="preserve">OpenVLA 7B (Prismatic VLM: DINOv2+SigLIP + Llama 2 7B), fine-tuned with OFT recipe; OFT+ adds FiLM</t>
   </si>
   <si>
@@ -244,90 +259,6 @@
     <t xml:space="preserve">https://arxiv.org/abs/2502.19645</t>
   </si>
   <si>
-    <t xml:space="preserve">FAST</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FAST: Efficient Action Tokenization for Vision-Language-Action Models</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Karl Pertsch (co-first with Kyle Stachowicz)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (2501.09747)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pi0-FAST: pi0 architecture on PaliGemma-3B (autoregressive 2B language backbone, no 300M flow expert); also applied to OpenVLA (Prismatic 7B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">autoregressive tokens: per-dimension quantile normalization -&gt; DCT -&gt; scale &amp; round (scale 10) -&gt; low-frequency-first flattening -&gt; BPE (vocab 1024); 1-second chunks (e.g., 15-step chunks on DROID at 15 Hz); ~30–60 tokens decoded per chunk</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compress action chunks into fewer, less-correlated tokens (DCT + BPE) to make autoregressive VLA training effective at high frequency; universal FAST+ tokenizer trained on ~1M 1-s action chunks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Training cost (fewer action tokens)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tokens per 1-s chunk naive vs FAST (Table I): BridgeV2 35-&gt;20 (1.75×), DROID 105-&gt;29 (3.6×), Bussing 140-&gt;28 (5.0×), Shirt fold 700-&gt;53 (13.2×). pi0-FAST matches diffusion pi0 'while reducing training time by up to 5x' (5× fewer GPU hours); ~3× fewer training steps on table bussing. Inference on NVIDIA 4090: pi0-FAST ~750 ms per chunk vs ~100 ms for diffusion pi0.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIBERO: comparable to diffusion pi0 (numbers only in figures; not extracted). Third-party (OpenVLA-OFT Table): pi0+FAST fine-tuned LIBERO S/O/G/L/avg 96.4/96.8/88.6/60.2/85.5. DROID zero-shot generalist policy (exact SR not in text).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smooth, highly correlated action signals compressible in frequency domain; BPE trained per dataset unless FAST+ used.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Training-efficiency gain comes at ~7.5× slower inference (~750 ms vs ~100 ms per chunk on 4090) due to autoregressive decoding of 30–60 tokens through the full backbone.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors: combining compression with non-autoregressive decoding (e.g., diffusion) left to future work; only static manipulators tested on hardware; slower inference made evaluation significantly slower. (reviewer inference) Effect on dynamic tasks requiring &lt;100 ms reaction.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2501.09747</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TinyVLA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TinyVLA: Towards Fast, Data-Efficient Vision-Language-Action Models for Robotic Manipulation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Junjie Wen (co-first with Yichen Zhu)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IEEE Robotics and Automation Letters (accepted Feb 2025, per PDF header) (2409.12514)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TinyVLA-S/B/H: 422M/740M/1.3B total, 101M/138M/143M trainable (Table II); Pythia language backbone in a small VLM (70M–1.4B family); 3B PaliGemma variant only in ablation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">diffusion: Diffusion Policy head conditioned via 3-layer MLP on VLM features (denoising steps and chunk size not stated in text read — UNVERIFIED)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Small VLM backbone (&lt;1.4B) + frozen VLM with LoRA on Q/K/V (5.0% of transformer params trainable) + diffusion head instead of autoregressive token decoding; no robot-data pretraining</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model size, latency, training data</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Table IV, single A6000, per-action prediction: TinyVLA-1B 14 ms vs OpenVLA-7B 292 ms (~20×) and OpenVLA-1B 140 ms (~10×).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meta-World 50 tasks avg: TinyVLA-H 31.6% vs Diffusion Policy 10.5%. Real Franka 5 tasks: TinyVLA-H 94.0% vs OpenVLA 68.3% (+25.7). Bimanual UR5: OpenVLA 0%; TinyVLA-H ~47.8% by Table III (text says 44.5%) vs DP 38.2%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VLM pretrained only on vision-language data is sufficient when fine-tuned on task demos; per-task/multi-task fine-tuning data available.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Smaller VLMs misinterpret instructions more often (0.4B variant); occasional failures under camera-view shift; OpenVLA slightly better on distant spatial generalization.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(reviewer inference) Denoising-step count and chunk size not reported, so latency is not directly comparable across papers; internal inconsistencies in text vs tables (21.5 vs 21.1 pts; 44.5 vs 47.8%). No dedicated limitations section.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2409.12514</t>
-  </si>
-  <si>
     <t xml:space="preserve">VLA-Cache</t>
   </si>
   <si>
@@ -340,6 +271,9 @@
     <t xml:space="preserve">NeurIPS 2025 (per PDF header) (2502.02175)</t>
   </si>
   <si>
+    <t xml:space="preserve">Reuses visual tokens across frames: the idea behind the stale-image variant (H1).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Applied to OpenVLA (7B), OpenVLA-OFT, CogACT (all Llama-2-based decoders)</t>
   </si>
   <si>
@@ -373,48 +307,6 @@
     <t xml:space="preserve">https://arxiv.org/abs/2502.02175</t>
   </si>
   <si>
-    <t xml:space="preserve">DeeR-VLA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DeeR-VLA: Dynamic Inference of Multimodal Large Language Models for Efficient Robot Execution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yang Yue (equal contribution with Yulin Wang)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NeurIPS 2024 (per PDF header) (2411.02359)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RoboFlamingo++ / OpenFlamingo, 3B (24 LLM layers) and 9B (32 layers) variants; multi-exit built on first 12 layers with 6 exit points; LSTM action head (window 12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">other: regression via LSTM action head on intermediate MLLM features (one action per step)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Dynamic early exit: LLM layers split into groups with exits; stop at first exit whose predicted action is consistent with previous exit's; per-exit thresholds tuned from demonstrations or online Bayesian optimization under average-FLOPs / peak-FLOPs / GPU-memory budgets</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compute, memory</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abstract: LLM computational cost reduced 5.2–6.5× and LLM GPU memory 2–6× 'without compromising performance'. LLM GFLOPs/action ~8.6–12.5 vs 31.2 baseline. On Nvidia V100: LLM inference 55 ms -&gt; 17.5 ms (ABCD-&gt;D; 68.1% reduction), without early-exit code optimization. Activated-LLM memory ~2 GB for DeeR-S (3B).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CALVIN avg successful length (DeeR / DeeR online / RoboFlamingo++): D-&gt;D 2.83/2.92/2.71; ABC-&gt;D 2.82/2.90/2.59; ABCD-&gt;D 4.13/4.13/4.07.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Many timesteps are 'easy' and need fewer layers; adjacent-exit action consistency is a valid confidence proxy; threshold calibration data or online interaction available.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requires training the multi-exit model (perceiver sampler + cross-attention fine-tuned, backbone frozen) — not training-free; savings limited to the LLM (vision encoder cost unchanged); variable per-step latency.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors: visual encoder cost also significant; experiments only on simulated benchmark (CALVIN). (reviewer inference) Worst-case latency guarantees for real-time control; applicability to chunked flow/diffusion VLAs.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2411.02359</t>
-  </si>
-  <si>
     <t xml:space="preserve">EfficientVLA</t>
   </si>
   <si>
@@ -427,6 +319,9 @@
     <t xml:space="preserve">arXiv (v1 'Preprint. Under review.'; later venue UNVERIFIED) (2506.10100)</t>
   </si>
   <si>
+    <t xml:space="preserve">Training-free acceleration with a small success loss: the same setting as this study.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Applied to CogACT 7.63B (DINOv2+SigLIP vision, Llama2-7B language module, Diffusion Transformer action head); pruned to 4.86B (L=22) or 5.87B (L=28)</t>
   </si>
   <si>
@@ -457,441 +352,252 @@
     <t xml:space="preserve">https://arxiv.org/abs/2506.10100</t>
   </si>
   <si>
-    <t xml:space="preserve">EfficientVLA-Survey</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A Survey on Efficient Vision-Language-Action Models</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zhaoshu Yu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (v3, 2026-09-28; no venue in comments field) (2510.24795)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A (survey)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A (survey; covers all paradigms)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Taxonomy of three pillars: (1) Efficient Model Design (efficient architectures and model compression); (2) Efficient Training (reducing computational burden during learning); (3) Efficient Data Collection (bottlenecks in acquiring and utilizing robot data)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model, training and data efficiency (taxonomy)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Claims to be the first comprehensive review of efficient VLAs across the model–training–data pipeline (authors' claim).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors summarize applications, key challenges and future directions (specific items not extracted — only the abstract page was read). Project page: https://evla-survey.github.io/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2510.24795</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DiffusionPolicy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diffusion Policy: Visuomotor Policy Learning via Action Diffusion</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cheng Chi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RSS 2023 (conference version); arXiv PDF read is the extended version (journal not named on the page) (2303.04137)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not a VLA (no language model). ResNet-18 vision encoder (~22M, trained end-to-end); CNN-based diffusion net ~22M (45M Transport) or time-series diffusion transformer ~9M (sim) / 80M (Kitchen, real Push-T)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">diffusion (DDPM, epsilon/noise-prediction MSE objective conditioned on observations); sim: 100 denoising iterations for training and inference; real: DDIM with 100 training / 10 inference iterations (Appendix A.4 says 16 — inconsistent); To=2, Tp=16, Ta=8 (receding-horizon control)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not an efficiency paper; DDIM reduces inference iterations (100 -&gt; 10) and action-sequence prediction with receding horizon amortizes inference over Ta=8 executed actions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">N/A (generative action-head reference)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">'0.1s inference latency on a Nvidia 3080 GPU' (DDIM, 10 inference iterations, real world)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Average improvement of 46.9% over prior methods (abstract of version read: 15 tasks from 4 benchmarks; Table 3: 12 tasks, 8 sim + 4 real). Third-party: LIBERO avg 72.4 (scratch) in OpenVLA-OFT/SmolVLA tables; Meta-World avg 10.5 in TinyVLA/SmolVLA tables.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sufficient task-specific demonstrations (behavior cloning); actions executed open-loop for Ta steps between replans; multimodal action distributions benefit from diffusion.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors: higher compute and inference latency than simpler methods such as LSTM-GMM; action-sequence prediction may not suffice for high-rate control tasks.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors: inherits behavior-cloning limits (poor with inadequate demos). (reviewer inference) Few-step / consistency distillation for faster sampling; scaling with language conditioning (addressed by later VLAs).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2303.04137</t>
+    <t xml:space="preserve">RTC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real-Time Execution of Action Chunking Flow Policies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NeurIPS 2025 (per PDF header) (2506.07339)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asynchronous execution of chunked flow policies: the alternative to re-planning at every step (H1).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied to pi0.5 (real world) and flow policies on Kinetix (sim); no new model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flow matching (base policy) with inference-time guided inpainting; n=5 denoising steps (sim and real); real: H=50, execution horizon s=25, 20 ms control period; sim: H=8, delays 0–4 steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Asynchronous execution without discontinuities: generate next chunk while current executes, freeze actions guaranteed to execute during inference delay, inpaint remaining actions via guidance with exponentially decaying soft mask; guidance weight clipped at β=5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency hiding (asynchronous execution)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Abstract: remains effective with inference delays &gt;300 ms (&gt;30% of prediction horizon). Real world (6 bimanual tasks, 480 episodes, injected +0/+100/+200 ms ≈ d 6/11/16): best average throughput at every delay, no degradation with delay (sync degrades ~linearly); same motion reported ~20% faster than synchronous (as extracted). Latency on RTX 4090 bf16: RTC 97 ms vs vanilla pi0.5 76 ms (per-denoising-step 14 -&gt; 35 ms due to backprop through each step); BID (N=16) 223 ms.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kinetix (12 dynamic tasks): RTC &gt; BID, naive async, temporal ensembling across delays (exact numbers in figures; not extracted). Real-world throughput gains significant at +100 and +200 ms.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base policy is diffusion/flow-based; inference delay d is known/estimated and smaller than the execution horizon; frozen prefix actions will actually be executed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training-free but adds ~21 ms (76 -&gt; 97 ms) per chunk from vector-Jacobian guidance; only for diffusion/flow policies; temporal ensembling fails (averages of valid actions not valid).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors: significant compute overhead; diffusion/flow only; not tested in more dynamic settings (e.g., legged locomotion). (reviewer inference) Interaction with step-reduction/distillation; A2C2 reports being orthogonal/complementary.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2506.07339</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RealtimeVLA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running VLAs at Real-time Speed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yunchao Ma</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arXiv (2510.26742)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CUDA graphs and kernel-level work for pi0: the graph lever of H2.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pi0-level VLA: PaliGemma backbone (SigLIP ~400M + Gemma 2.6B, ~3B) + ~300M action expert.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flow matching, 10 action-expert denoising steps (pi0 recipe).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inference-only systems optimisation: CUDA graphs to remove CPU launch overhead (~2x), folding RMSNorm affine and the action-time embedding into adjacent linear layers, fused QKV/RoPE, fused gated linear layers and scalar ops, Triton GEMM tile tuning, dropping the last LLM layer (17 of 18); plus a streaming inference framework.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency (CPU launch overhead, kernel fusion)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTX 4090, bf16, 10 steps (Table 1): 2 views 106.5 ms (naive torch) / 53.7 ms (openpi JAX) -&gt; 27.3 ms; 1 view 20.0 ms; 3 views 36.8 ms; 30 Hz frame rate.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real-world falling-pen catching: 10/10 consecutive successes (policy trained with openpi on 600 episodes). No standard benchmark reported.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model weights fixed; a single consumer GPU with native bf16; per-shape kernel tuning for one model and input size.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Large engineering effort (hand-written/fused kernels) tied to one architecture and GPU; dropping a layer changes the model; no closed-loop success comparison against the unoptimised policy.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(reviewer inference) Whether each fused/approximated step leaves closed-loop success unchanged on a standard benchmark; portability to GPUs without bf16 tensor cores.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes (speed-ups); the task policy itself was trained</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2510.26742</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Coda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fewer Steps, Better Actions: Rethinking Flow-Matching Inference for VLA Policies</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zhipeng Tang</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arXiv (2609.21216)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fewer flow steps for pi0.5 (3 steps hold, 1 step drops): the step lever of H2 and its contrast.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Frozen pi0.5 (fine-tuned) and frozen official SmolVLA; corrector parameter count UNVERIFIED (not reported).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flow matching with few Euler steps + a learned endpoint correction (lightweight Transformer reading the candidate action, the source noise and the shared prefix cache).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Spend part of the integration budget on a learned residual corrector instead of more flow steps.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency (fewer flow steps + learned correction)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pi0.5-FT on A100: 10 steps 233.0 ms -&gt; Coda 2 steps 109.9 ms (2.12x); SmolVLA: 233.5 -&gt; 118.1 ms (1.98x).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RoboTwin Easy (50 tasks), pi0.5-FT naive steps 1/2/3/5/10: 59.76/67.40/71.28/71.64/71.52%; Coda 2 steps 71.88%. SmolVLA (10 tasks) naive 1/2/5/10: 35.0/60.8/60.8/64.4%; Coda 2 steps 69.4%.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Demonstrations available to train the corrector (SmolVLA: 18,716 steps, batch 256); base policy frozen.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requires training and a second network; naive step reduction alone is nearly free for pi0.5 down to 3 steps but collapses at 1 step (and for SmolVLA at 1 step).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(reviewer inference) Results are on RoboTwin; whether the same step curve holds on LIBERO and for per-step re-planning.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">no (corrector only)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2609.21216</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Islam-ONNX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When Faster VLA Deployment Changes Closed-Loop Behavior: Task Success-Latency Analysis of SmolVLA Across PyTorch and ONNX Variants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rafiqul Islam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arXiv (2609.14146)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faster deployment of this very checkpoint lowered success (70% to 41%): motivates paired tests.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Same checkpoint as this study: HuggingFaceVLA/smolvla_libero, LeRobot 0.6.1 (MuJoCo 3.3.2).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flow matching, 10 flow steps (released configuration).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Runtime change: PyTorch+AMP vs ONNX Runtime (CUDA EP) with 'requested' FP16/INT8 exports; static language width 16/24/32 tokens.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Latency (runtime/export), closed-loop side effects</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTX 2060 6 GB, batch 1: PyTorch+AMP p50 903 ms / p99 1181 ms; ONNX p50 537.5-549.2 ms (p99 532-601 ms) - about 2x lower latency.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIBERO Spatial / Object, 100 episodes each: PyTorch+AMP 70.0 / 88.0; ONNX width 16 41.0 / 89.0; width 24 75.0 / 90.0; width 32 71.0 / 87.0. Paired 300 episodes, Spatial: 56.7 vs 33.0 (McNemar p = 2.2e-9).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One GPU, one checkpoint, one seed; the exported graph has a static language width (width 16 truncates 5 of 10 Spatial instructions).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Faster runtime but a silent behaviour change: truncated instructions cut Spatial success by ~29 pp; the 'INT8' artifact is a byte-identical FP32 graph, i.e. not real INT8.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Authors: factors other than width (graph conversion, AMP vs FP32, kernels, true INT8, TensorRT) not isolated; no equivalence test ('a non-significant two-proportion test is not an equivalence result').</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://arxiv.org/abs/2609.14146</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generative family</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Network predicts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training objective</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Time / noise-level sampling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inference sampler &amp; steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What each step re-runs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chunk / executed actions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reported latency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Source</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diffusion Policy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diffusion (DDPM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Noise eps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSE(eps, eps_theta(O, A^0 + eps_k, k))</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Uniform over 100 DDPM steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sim: 100 DDPM steps; real: DDIM 10 steps (App. A.4 says 16)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Full denoising network (~9-80M)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tp=16 predicted, Ta=8 executed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1 s on RTX 3080 (DDIM 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">arxiv.org/abs/2303.04137</t>
   </si>
   <si>
     <t xml:space="preserve">CogACT</t>
   </si>
   <si>
-    <t xml:space="preserve">CogACT: A Foundational Vision-Language-Action Model for Synergizing Cognition and Action in Robotic Manipulation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Qixiu Li</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (v1, 29 Nov 2024; venue not stated) (2411.19650)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.6B total (abstract: 7B): DINOv2+SigLIP -&gt; 256 visual tokens, LLaMA-2 language backbone, learnable cognition token; DiT action module Small 13M / Base 89M (default) / Large 308M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">diffusion: DiT action module conditioned on the VLM cognition feature (cognition feature + noisy action tokens as transformer inputs; denoising step added to cognition feature via sinusoidal encoding); noise-prediction MSE; DDIM 10 inference steps, CFG scale 1.5; predicts current + 15 future actions (16); Adaptive Action Ensemble (α=0.1, C=0.2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Not an efficiency paper; decouples cognition (single feature from 7B VLM) from action generation in a small DiT so multi-step denoising does not re-run the VLM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Compute (VLM runs once, small DiT denoises)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inference latency not reported in the paper (A6000/A100 used for sim). Third-party: VLA-Cache measures CogACT 54.29 ms on RTX 4090 (SIMPLER VM); EfficientVLA measures 0.2342 s/step on A40.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SIMPLER: Google VM 74.8 / VA 61.3 / WidowX VM 51.3 (OpenVLA 34.3/39.3/4.2; RT-2-X 46.3/54.4/–; Octo-Base 11.0/1.2/17.5). Abstract: &gt;35% over OpenVLA in sim, +18% abs over RT-2-X (55B), &gt;55% over OpenVLA on real robots. Realman seen 71.2% vs 12.1%; Franka 61.4% vs 6.8%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A single cognition feature carries sufficient task information for action generation; training on single-arm end-effector OXE subsets with third-person camera.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.6B total still large; 10 DDIM steps + CFG (1.5) per inference; action ensemble adds temporal smoothing at cost of reactivity (reviewer inference).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(reviewer inference) Latency not reported; weaker on unseen categories (25.0% on Realman unseen-category task); small evaluation sample (e.g., 11 Franka trials/task); no dedicated limitations section.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2411.19650</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A2C2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Leave No Observation Behind: Real-time Correction for VLA Action Chunks</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kohei Sendai</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (v1, 27 Sep 2025; no venue in comments field) (2509.23224)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Base: SmolVLA (450M, trained from scratch on LIBERO because pretrained embodiment differs) for LIBERO; flow policy for Kinetix. Correction head: ~32M for LIBERO (6-layer transformer encoder + 3-layer MLP), ~0.31M for Kinetix (3-layer MLP, 512 hidden)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">other: base VLA action chunk (SmolVLA flow matching) + per-step residual correction from a lightweight head conditioned on latest observation, base action, sinusoidal in-chunk index feature, base-policy latent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Restore closed-loop reactivity of chunked/asynchronous execution without re-running the large VLA: small correction head runs every control step; orthogonal to RTC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reactivity of chunked/asynchronous execution</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NVIDIA RTX 5080 laptop GPU (16 GB), mean of 100 trials: SmolVLA ~101 ms per inference vs A2C2 head ~4.7 ms per step. Abstract: '+23% point' (Kinetix, 12 tasks) and '+7% point' (LIBERO Spatial) vs RTC.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIBERO-Spatial, SmolVLA naive async -&gt; +A2C2 (Table 7; e=exec horizon, d=delay): e40/d10 67-&gt;84; e40/d5 66-&gt;86; e40/d3 65-&gt;86; e40/d1 74-&gt;83; e10/d10 75-&gt;88; e10/d5 82-&gt;92; e10/d3 81-&gt;89; e10/d1 83-&gt;92; e50/d0 71-&gt;84; e40/d0 79-&gt;89; e30/d0 79-&gt;89; e10/d0 85-&gt;87; e5/d0 83-&gt;85; e1/d0 77-&gt;84. Table 1 gives different values for same settings (e10/d0 81.8-&gt;89.2; e40/d10 64.4-&gt;84.2; e50/d0 72.2-&gt;81.6). Kinetix: &gt;85% at d=4 even at horizon 7.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Correction head trained post hoc on the same demonstrations using cached base-policy outputs; no retraining of base VLA; access to base-policy latent features.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requires training a (small) extra head per task/embodiment — not training-free; adds ~4.7 ms per control step; LIBERO base SmolVLA trained from scratch (not the pretrained checkpoint); head training sensitive to LR (1e-4 did not work well).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors: scalability to richer language, OOD settings and more dynamic tasks beyond LIBERO-Spatial needs validation. (reviewer inference) LIBERO tables report no RTC column although abstract claims +7 pts vs RTC on LIBERO Spatial; Table 1 vs Table 7 inconsistent; note SmolVLA naive SR is non-monotonic in e (best e=10, d=0: 85%), consistent with SmolVLA's own chunk-size ablation favoring 10.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2509.23224</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RTC</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real-Time Execution of Action Chunking Flow Policies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NeurIPS 2025 (per PDF header) (2506.07339)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Applied to pi0.5 (real world) and flow policies on Kinetix (sim); no new model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">flow matching (base policy) with inference-time guided inpainting; n=5 denoising steps (sim and real); real: H=50, execution horizon s=25, 20 ms control period; sim: H=8, delays 0–4 steps</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Asynchronous execution without discontinuities: generate next chunk while current executes, freeze actions guaranteed to execute during inference delay, inpaint remaining actions via guidance with exponentially decaying soft mask; guidance weight clipped at β=5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latency hiding (asynchronous execution)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Abstract: remains effective with inference delays &gt;300 ms (&gt;30% of prediction horizon). Real world (6 bimanual tasks, 480 episodes, injected +0/+100/+200 ms ≈ d 6/11/16): best average throughput at every delay, no degradation with delay (sync degrades ~linearly); same motion reported ~20% faster than synchronous (as extracted). Latency on RTX 4090 bf16: RTC 97 ms vs vanilla pi0.5 76 ms (per-denoising-step 14 -&gt; 35 ms due to backprop through each step); BID (N=16) 223 ms.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kinetix (12 dynamic tasks): RTC &gt; BID, naive async, temporal ensembling across delays (exact numbers in figures; not extracted). Real-world throughput gains significant at +100 and +200 ms.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Base policy is diffusion/flow-based; inference delay d is known/estimated and smaller than the execution horizon; frozen prefix actions will actually be executed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Training-free but adds ~21 ms (76 -&gt; 97 ms) per chunk from vector-Jacobian guidance; only for diffusion/flow policies; temporal ensembling fails (averages of valid actions not valid).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors: significant compute overhead; diffusion/flow only; not tested in more dynamic settings (e.g., legged locomotion). (reviewer inference) Interaction with step-reduction/distillation; A2C2 reports being orthogonal/complementary.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2506.07339</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RealtimeVLA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Running VLAs at Real-time Speed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Yunchao Ma</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (2510.26742)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pi0-level VLA: PaliGemma backbone (SigLIP ~400M + Gemma 2.6B, ~3B) + ~300M action expert.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">flow matching, 10 action-expert denoising steps (pi0 recipe).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inference-only systems optimisation: CUDA graphs to remove CPU launch overhead (~2x), folding RMSNorm affine and the action-time embedding into adjacent linear layers, fused QKV/RoPE, fused gated linear layers and scalar ops, Triton GEMM tile tuning, dropping the last LLM layer (17 of 18); plus a streaming inference framework.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latency (CPU launch overhead, kernel fusion)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RTX 4090, bf16, 10 steps (Table 1): 2 views 106.5 ms (naive torch) / 53.7 ms (openpi JAX) -&gt; 27.3 ms; 1 view 20.0 ms; 3 views 36.8 ms; 30 Hz frame rate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Real-world falling-pen catching: 10/10 consecutive successes (policy trained with openpi on 600 episodes). No standard benchmark reported.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model weights fixed; a single consumer GPU with native bf16; per-shape kernel tuning for one model and input size.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Large engineering effort (hand-written/fused kernels) tied to one architecture and GPU; dropping a layer changes the model; no closed-loop success comparison against the unoptimised policy.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(reviewer inference) Whether each fused/approximated step leaves closed-loop success unchanged on a standard benchmark; portability to GPUs without bf16 tensor cores.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yes (speed-ups); the task policy itself was trained</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2510.26742</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Islam-ONNX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">When Faster VLA Deployment Changes Closed-Loop Behavior: Task Success-Latency Analysis of SmolVLA Across PyTorch and ONNX Variants</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rafiqul Islam</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (2609.14146)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Same checkpoint as this study: HuggingFaceVLA/smolvla_libero, LeRobot 0.6.1 (MuJoCo 3.3.2).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">flow matching, 10 flow steps (released configuration).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime change: PyTorch+AMP vs ONNX Runtime (CUDA EP) with 'requested' FP16/INT8 exports; static language width 16/24/32 tokens.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latency (runtime/export), closed-loop side effects</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RTX 2060 6 GB, batch 1: PyTorch+AMP p50 903 ms / p99 1181 ms; ONNX p50 537.5-549.2 ms (p99 532-601 ms) - about 2x lower latency.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIBERO Spatial / Object, 100 episodes each: PyTorch+AMP 70.0 / 88.0; ONNX width 16 41.0 / 89.0; width 24 75.0 / 90.0; width 32 71.0 / 87.0. Paired 300 episodes, Spatial: 56.7 vs 33.0 (McNemar p = 2.2e-9).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">One GPU, one checkpoint, one seed; the exported graph has a static language width (width 16 truncates 5 of 10 Spatial instructions).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Faster runtime but a silent behaviour change: truncated instructions cut Spatial success by ~29 pp; the 'INT8' artifact is a byte-identical FP32 graph, i.e. not real INT8.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Authors: factors other than width (graph conversion, AMP vs FP32, kernels, true INT8, TensorRT) not isolated; no equivalence test ('a non-significant two-proportion test is not an equivalence result').</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2609.14146</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Coda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fewer Steps, Better Actions: Rethinking Flow-Matching Inference for VLA Policies</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Zhipeng Tang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (2609.21216)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Frozen pi0.5 (fine-tuned) and frozen official SmolVLA; corrector parameter count UNVERIFIED (not reported).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">flow matching with few Euler steps + a learned endpoint correction (lightweight Transformer reading the candidate action, the source noise and the shared prefix cache).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Spend part of the integration budget on a learned residual corrector instead of more flow steps.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latency (fewer flow steps + learned correction)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pi0.5-FT on A100: 10 steps 233.0 ms -&gt; Coda 2 steps 109.9 ms (2.12x); SmolVLA: 233.5 -&gt; 118.1 ms (1.98x).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RoboTwin Easy (50 tasks), pi0.5-FT naive steps 1/2/3/5/10: 59.76/67.40/71.28/71.64/71.52%; Coda 2 steps 71.88%. SmolVLA (10 tasks) naive 1/2/5/10: 35.0/60.8/60.8/64.4%; Coda 2 steps 69.4%.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Demonstrations available to train the corrector (SmolVLA: 18,716 steps, batch 256); base policy frozen.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Requires training and a second network; naive step reduction alone is nearly free for pi0.5 down to 3 steps but collapses at 1 step (and for SmolVLA at 1 step).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(reviewer inference) Results are on RoboTwin; whether the same step curve holds on LIBERO and for per-step re-planning.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">no (corrector only)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2609.21216</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vla.cpp</t>
-  </si>
-  <si>
-    <t xml:space="preserve">vla.cpp: A Unified Inference Runtime for Vision-Language-Action Models</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Khanh D. Nguyen</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arXiv (2606.08094)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C++ runtime for eleven VLA models (list UNVERIFIED from the abstract); SmolVLA and BitVLA discussed.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Architecture-specific heads; iterative policies reuse observation-dependent computation across solver steps.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Runtime without PyTorch: shared loading/execution/serving; ternary tensor-core kernel for BitVLA.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Latency, memory, edge deployment (runtime)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BitVLA client inference 4.0-4.6x faster than a CUDA-core baseline on RTX 3060 and AGX Orin.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIBERO-Object: BitVLA 200/200 episodes on an 8 GB Jetson Orin Nano; a SmolVLA case study links positional-index precision to gripper commands and task success.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Re-implementation of each model in C++ matches the reference behaviour.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Engineering cost per architecture; numerical details (e.g. positional-index precision) can change closed-loop behaviour.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(reviewer inference) Absolute latencies and SmolVLA success rates not given in the abstract.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://arxiv.org/abs/2606.08094</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Model</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generative family</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Network predicts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Training objective</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Time / noise-level sampling</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Inference sampler &amp; steps</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What each step re-runs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Chunk / executed actions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reported latency</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Source</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diffusion Policy</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diffusion (DDPM)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Noise eps</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MSE(eps, eps_theta(O, A^0 + eps_k, k))</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Uniform over 100 DDPM steps</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sim: 100 DDPM steps; real: DDIM 10 steps (App. A.4 says 16)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Full denoising network (~9-80M)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tp=16 predicted, Ta=8 executed</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.1 s on RTX 3080 (DDIM 10)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">arxiv.org/abs/2303.04137</t>
-  </si>
-  <si>
     <t xml:space="preserve">Diffusion (DiT action module)</t>
   </si>
   <si>
@@ -1126,10 +832,10 @@
     <t xml:space="preserve">How this matrix was built: every entry was read from the paper's own arXiv abstract, HTML or PDF (column 'Source'). 'UNVERIFIED' marks values not found in the text that was read; '(reviewer inference)' marks open questions that are the reviewer's reading, not the authors' statement.</t>
   </si>
   <si>
-    <t xml:space="preserve">Inconsistencies found in the sources: Diffusion Policy states 10 DDIM inference steps (Sec. 3.4) and 16 (App. A.4); VLA-Cache's 1.7x headline is larger than its per-model tables (OpenVLA 1.63x); TinyVLA text and tables differ (44.5% vs 47.8%); A2C2 Table 1 and Table 7 differ for the same settings and its LIBERO tables contain no RTC column.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A2C2 trains its own SmolVLA from scratch on LIBERO; its execution-horizon results (e=5: 0.83 &gt; e=1: 0.77) are not for the checkpoint used in this study, for which executing 5 actions per re-plan lowers SR by 12.5 pp.</t>
+    <t xml:space="preserve">Inconsistencies found in the sources: Diffusion Policy states 10 DDIM inference steps (Sec. 3.4) and 16 (App. A.4); VLA-Cache's 1.7x headline is larger than its per-model tables (OpenVLA 1.63x).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Scope: the matrix keeps the ten papers that are most cited and most directly tied to this study (column 'Relevance to this study'). Also read, and cited in the report where used, but left out to keep the matrix focused: OpenVLA, FAST, TinyVLA, DeeR-VLA, CogACT, A2C2, an efficient-VLA survey and vla.cpp. Of these, A2C2 matters most for H1: it trains its own SmolVLA from scratch on LIBERO, and its execution-horizon results (e=5: 0.83 &gt; e=1: 0.77) do not transfer to the checkpoint used here, where executing 5 actions per re-plan lowers SR by 12.5 pp.</t>
   </si>
   <si>
     <t xml:space="preserve">Islam (2026) uses the same checkpoint and LeRobot version on a Turing GPU (RTX 2060): its PyTorch+AMP Spatial success (70.0%, 100 episodes) is in the range of this study's baseline (77.0%, 200 episodes); its ONNX speed-up came with a behaviour change (truncated instructions), which motivates checking closed-loop equivalence for every efficiency change.</t>
@@ -1138,7 +844,7 @@
     <t xml:space="preserve">Coda (2026) and Realtime-VLA (2025) already apply fewer flow steps and CUDA graphs, respectively; this study does not claim these levers as new.</t>
   </si>
   <si>
-    <t xml:space="preserve">Venues for pi0, OpenVLA and OpenVLA-OFT are not stated on the arXiv pages read and are left as arXiv.</t>
+    <t xml:space="preserve">Venues for pi0 and OpenVLA-OFT are not stated on the arXiv pages read and are left as arXiv.</t>
   </si>
 </sst>
 </file>
@@ -1629,7 +1335,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
@@ -1637,14 +1343,15 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="6" style="0" width="34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="10" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="12" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="13" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1696,905 +1403,538 @@
       <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>2025</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="O2" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
+      </c>
+      <c r="Q2" s="3" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D3" s="5" t="n">
         <v>2024</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="K3" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="L3" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="M3" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="N3" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="O3" s="5" t="s">
-        <v>29</v>
+        <v>46</v>
       </c>
       <c r="P3" s="5" t="s">
-        <v>44</v>
+        <v>31</v>
+      </c>
+      <c r="Q3" s="5" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D4" s="3" t="n">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>58</v>
+        <v>31</v>
+      </c>
+      <c r="Q4" s="3" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>2025</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="K5" s="5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="L5" s="5" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="M5" s="5" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="N5" s="5" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="O5" s="5" t="s">
-        <v>29</v>
+        <v>76</v>
       </c>
       <c r="P5" s="5" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>31</v>
+      </c>
+      <c r="Q5" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="D6" s="3" t="n">
         <v>2025</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="N6" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="O6" s="3" t="s">
-        <v>29</v>
+        <v>91</v>
       </c>
       <c r="P6" s="3" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>92</v>
+      </c>
+      <c r="Q6" s="3" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="G7" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="H7" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I7" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J7" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="K7" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="L7" s="5" t="s">
+        <v>104</v>
+      </c>
+      <c r="M7" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="N7" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="O7" s="5" t="s">
+        <v>107</v>
+      </c>
+      <c r="P7" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>94</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>95</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="L7" s="5" t="s">
-        <v>97</v>
-      </c>
-      <c r="M7" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="N7" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="O7" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="P7" s="5" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="Q7" s="5" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>103</v>
+        <v>35</v>
       </c>
       <c r="D8" s="3" t="n">
         <v>2025</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="N8" s="3" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="O8" s="3" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="P8" s="3" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>92</v>
+      </c>
+      <c r="Q8" s="3" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="I9" s="5" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="J9" s="5" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="K9" s="5" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="L9" s="5" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="M9" s="5" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="N9" s="5" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="O9" s="5" t="s">
-        <v>29</v>
+        <v>136</v>
       </c>
       <c r="P9" s="5" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>137</v>
+      </c>
+      <c r="Q9" s="5" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="2" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>133</v>
+        <v>142</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>134</v>
+        <v>143</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>136</v>
+        <v>145</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>137</v>
+        <v>146</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>138</v>
+        <v>147</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>140</v>
+        <v>149</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>141</v>
+        <v>150</v>
       </c>
       <c r="N10" s="3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="O10" s="3" t="s">
-        <v>114</v>
+        <v>152</v>
       </c>
       <c r="P10" s="3" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>153</v>
+      </c>
+      <c r="Q10" s="3" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="I11" s="5" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="K11" s="5" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="L11" s="5" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="M11" s="5" t="s">
-        <v>153</v>
+        <v>166</v>
       </c>
       <c r="N11" s="5" t="s">
-        <v>154</v>
+        <v>167</v>
       </c>
       <c r="O11" s="5" t="s">
-        <v>29</v>
+        <v>168</v>
       </c>
       <c r="P11" s="5" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="74.6" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
-        <v>156</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>158</v>
-      </c>
-      <c r="D12" s="3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>159</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>160</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>162</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>163</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>165</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>166</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P12" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="Q11" s="5" t="s">
         <v>169</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="85.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>171</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>172</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>2024</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>173</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>174</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>175</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>176</v>
-      </c>
-      <c r="I13" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="J13" s="5" t="s">
-        <v>178</v>
-      </c>
-      <c r="K13" s="5" t="s">
-        <v>179</v>
-      </c>
-      <c r="L13" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="M13" s="5" t="s">
-        <v>181</v>
-      </c>
-      <c r="N13" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="O13" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="P13" s="5" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
-        <v>184</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>185</v>
-      </c>
-      <c r="C14" s="3" t="s">
-        <v>186</v>
-      </c>
-      <c r="D14" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>187</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>188</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>189</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>190</v>
-      </c>
-      <c r="I14" s="3" t="s">
-        <v>191</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>192</v>
-      </c>
-      <c r="K14" s="3" t="s">
-        <v>193</v>
-      </c>
-      <c r="L14" s="3" t="s">
-        <v>194</v>
-      </c>
-      <c r="M14" s="3" t="s">
-        <v>195</v>
-      </c>
-      <c r="N14" s="3" t="s">
-        <v>196</v>
-      </c>
-      <c r="O14" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="P14" s="3" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="4" t="s">
-        <v>198</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>199</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="5" t="n">
-        <v>2025</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>200</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>201</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="I15" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="J15" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="K15" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="L15" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="M15" s="5" t="s">
-        <v>208</v>
-      </c>
-      <c r="N15" s="5" t="s">
-        <v>209</v>
-      </c>
-      <c r="O15" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="P15" s="5" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="64.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2" t="s">
-        <v>211</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>212</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>213</v>
-      </c>
-      <c r="D16" s="3" t="n">
-        <v>2025</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>215</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>216</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>217</v>
-      </c>
-      <c r="I16" s="3" t="s">
-        <v>218</v>
-      </c>
-      <c r="J16" s="3" t="s">
-        <v>219</v>
-      </c>
-      <c r="K16" s="3" t="s">
-        <v>220</v>
-      </c>
-      <c r="L16" s="3" t="s">
-        <v>221</v>
-      </c>
-      <c r="M16" s="3" t="s">
-        <v>222</v>
-      </c>
-      <c r="N16" s="3" t="s">
-        <v>223</v>
-      </c>
-      <c r="O16" s="3" t="s">
-        <v>224</v>
-      </c>
-      <c r="P16" s="3" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>228</v>
-      </c>
-      <c r="D17" s="5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>229</v>
-      </c>
-      <c r="F17" s="5" t="s">
-        <v>230</v>
-      </c>
-      <c r="G17" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="H17" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="I17" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="J17" s="5" t="s">
-        <v>234</v>
-      </c>
-      <c r="K17" s="5" t="s">
-        <v>235</v>
-      </c>
-      <c r="L17" s="5" t="s">
-        <v>236</v>
-      </c>
-      <c r="M17" s="5" t="s">
-        <v>237</v>
-      </c>
-      <c r="N17" s="5" t="s">
-        <v>238</v>
-      </c>
-      <c r="O17" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="P17" s="5" t="s">
-        <v>239</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
-        <v>240</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>241</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>242</v>
-      </c>
-      <c r="D18" s="3" t="n">
-        <v>2026</v>
-      </c>
-      <c r="E18" s="3" t="s">
-        <v>243</v>
-      </c>
-      <c r="F18" s="3" t="s">
-        <v>244</v>
-      </c>
-      <c r="G18" s="3" t="s">
-        <v>245</v>
-      </c>
-      <c r="H18" s="3" t="s">
-        <v>246</v>
-      </c>
-      <c r="I18" s="3" t="s">
-        <v>247</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>248</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>249</v>
-      </c>
-      <c r="L18" s="3" t="s">
-        <v>250</v>
-      </c>
-      <c r="M18" s="3" t="s">
-        <v>251</v>
-      </c>
-      <c r="N18" s="3" t="s">
-        <v>252</v>
-      </c>
-      <c r="O18" s="3" t="s">
-        <v>253</v>
-      </c>
-      <c r="P18" s="3" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="4" t="s">
-        <v>255</v>
-      </c>
-      <c r="B19" s="5" t="s">
-        <v>256</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>2026</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>258</v>
-      </c>
-      <c r="F19" s="5" t="s">
-        <v>259</v>
-      </c>
-      <c r="G19" s="5" t="s">
-        <v>260</v>
-      </c>
-      <c r="H19" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="I19" s="5" t="s">
-        <v>262</v>
-      </c>
-      <c r="J19" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="K19" s="5" t="s">
-        <v>264</v>
-      </c>
-      <c r="L19" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="M19" s="5" t="s">
-        <v>266</v>
-      </c>
-      <c r="N19" s="5" t="s">
-        <v>267</v>
-      </c>
-      <c r="O19" s="5" t="s">
-        <v>114</v>
-      </c>
-      <c r="P19" s="5" t="s">
-        <v>268</v>
       </c>
     </row>
   </sheetData>
@@ -2629,204 +1969,204 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>269</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>270</v>
+        <v>171</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>271</v>
+        <v>172</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>272</v>
+        <v>173</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>273</v>
+        <v>174</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>274</v>
+        <v>175</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>275</v>
+        <v>176</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>276</v>
+        <v>177</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>277</v>
+        <v>178</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>278</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>279</v>
+        <v>180</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>280</v>
+        <v>181</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>281</v>
+        <v>182</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>282</v>
+        <v>183</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>283</v>
+        <v>184</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>284</v>
+        <v>185</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>285</v>
+        <v>186</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>286</v>
+        <v>187</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>287</v>
+        <v>188</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>288</v>
+        <v>189</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>170</v>
+        <v>190</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>289</v>
+        <v>191</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>281</v>
+        <v>182</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>290</v>
+        <v>192</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>291</v>
+        <v>193</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>292</v>
+        <v>194</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>293</v>
+        <v>195</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>294</v>
+        <v>196</v>
       </c>
       <c r="I3" s="5" t="s">
-        <v>295</v>
+        <v>197</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>296</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>297</v>
+        <v>199</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>298</v>
+        <v>200</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>299</v>
+        <v>201</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>300</v>
+        <v>202</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>301</v>
+        <v>203</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>302</v>
+        <v>204</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>303</v>
+        <v>205</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>304</v>
+        <v>206</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>305</v>
+        <v>207</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>306</v>
+        <v>208</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>297</v>
+        <v>199</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>307</v>
+        <v>209</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>308</v>
+        <v>210</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>309</v>
+        <v>211</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>310</v>
+        <v>212</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>311</v>
+        <v>213</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>312</v>
+        <v>214</v>
       </c>
       <c r="I5" s="5" t="s">
-        <v>313</v>
+        <v>215</v>
       </c>
       <c r="J5" s="5" t="s">
-        <v>314</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>315</v>
+        <v>217</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>316</v>
+        <v>218</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>317</v>
+        <v>219</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>318</v>
+        <v>220</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>319</v>
+        <v>221</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>320</v>
+        <v>222</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>321</v>
+        <v>223</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>322</v>
+        <v>224</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>323</v>
+        <v>225</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>324</v>
+        <v>226</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>325</v>
+        <v>227</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>326</v>
+        <v>228</v>
       </c>
       <c r="B9" s="7"/>
       <c r="C9" s="7"/>
@@ -2840,7 +2180,7 @@
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>327</v>
+        <v>229</v>
       </c>
       <c r="B10" s="7"/>
       <c r="C10" s="7"/>
@@ -2854,7 +2194,7 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>328</v>
+        <v>230</v>
       </c>
       <c r="B11" s="7"/>
       <c r="C11" s="7"/>
@@ -2868,7 +2208,7 @@
     </row>
     <row r="12" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>329</v>
+        <v>231</v>
       </c>
       <c r="B12" s="7"/>
       <c r="C12" s="7"/>
@@ -2915,41 +2255,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>330</v>
+        <v>232</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>331</v>
+        <v>233</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>332</v>
+        <v>234</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>333</v>
+        <v>235</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>334</v>
+        <v>236</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>335</v>
+        <v>237</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>336</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>337</v>
+        <v>239</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>338</v>
+        <v>240</v>
       </c>
       <c r="C4" s="10" t="n">
         <v>10</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E4" s="11" t="n">
         <v>789.2</v>
@@ -2961,16 +2301,16 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="9" t="s">
-        <v>339</v>
+        <v>241</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>338</v>
+        <v>240</v>
       </c>
       <c r="C5" s="10" t="n">
         <v>3</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E5" s="11" t="n">
         <v>432.7</v>
@@ -2982,16 +2322,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="9" t="s">
-        <v>340</v>
+        <v>242</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>338</v>
+        <v>240</v>
       </c>
       <c r="C6" s="10" t="n">
         <v>10</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="E6" s="11" t="n">
         <v>572</v>
@@ -3003,16 +2343,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>341</v>
+        <v>243</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>341</v>
+        <v>243</v>
       </c>
       <c r="C7" s="10" t="n">
         <v>10</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E7" s="11" t="n">
         <v>616.1</v>
@@ -3024,16 +2364,16 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>342</v>
+        <v>244</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>341</v>
+        <v>243</v>
       </c>
       <c r="C8" s="10" t="n">
         <v>10</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>178</v>
@@ -3045,16 +2385,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>343</v>
+        <v>245</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>341</v>
+        <v>243</v>
       </c>
       <c r="C9" s="10" t="n">
         <v>3</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E9" s="11" t="n">
         <v>245.2</v>
@@ -3066,16 +2406,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>344</v>
+        <v>246</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>341</v>
+        <v>243</v>
       </c>
       <c r="C10" s="10" t="n">
         <v>3</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="E10" s="11" t="n">
         <v>111.9</v>
@@ -3087,16 +2427,16 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>345</v>
+        <v>247</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>341</v>
+        <v>243</v>
       </c>
       <c r="C11" s="10" t="n">
         <v>2</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="E11" s="11" t="n">
         <v>103.2</v>
@@ -3108,16 +2448,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>346</v>
+        <v>248</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>341</v>
+        <v>243</v>
       </c>
       <c r="C12" s="10" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>114</v>
+        <v>92</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>93.3</v>
@@ -3129,38 +2469,38 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>347</v>
+        <v>249</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>348</v>
+        <v>250</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>349</v>
+        <v>251</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>350</v>
+        <v>252</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>351</v>
+        <v>253</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>352</v>
+        <v>254</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>353</v>
+        <v>255</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>354</v>
+        <v>256</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>355</v>
+        <v>257</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="s">
-        <v>356</v>
+        <v>258</v>
       </c>
       <c r="B17" s="14" t="n">
         <v>500</v>
@@ -3180,7 +2520,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>357</v>
+        <v>259</v>
       </c>
       <c r="B18" s="14" t="n">
         <v>200</v>
@@ -3206,7 +2546,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="s">
-        <v>343</v>
+        <v>245</v>
       </c>
       <c r="B19" s="14" t="n">
         <v>500</v>
@@ -3232,7 +2572,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="9" t="s">
-        <v>358</v>
+        <v>260</v>
       </c>
       <c r="B20" s="14" t="n">
         <v>200</v>
@@ -3258,7 +2598,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
-        <v>359</v>
+        <v>261</v>
       </c>
       <c r="B21" s="14" t="n">
         <v>200</v>
@@ -3284,7 +2624,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
-        <v>360</v>
+        <v>262</v>
       </c>
       <c r="B22" s="14" t="n">
         <v>200</v>
@@ -3310,7 +2650,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
-        <v>361</v>
+        <v>263</v>
       </c>
       <c r="B23" s="14" t="n">
         <v>200</v>
@@ -3336,7 +2676,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
-        <v>362</v>
+        <v>264</v>
       </c>
       <c r="B24" s="14" t="n">
         <v>200</v>
@@ -3362,7 +2702,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="9" t="s">
-        <v>363</v>
+        <v>265</v>
       </c>
       <c r="B25" s="14" t="n">
         <v>500</v>
@@ -3388,7 +2728,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="9" t="s">
-        <v>364</v>
+        <v>266</v>
       </c>
       <c r="B26" s="14" t="n">
         <v>200</v>
@@ -3414,7 +2754,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>365</v>
+        <v>267</v>
       </c>
     </row>
   </sheetData>
@@ -3441,32 +2781,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="19" t="s">
-        <v>366</v>
+        <v>268</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="19" t="s">
-        <v>367</v>
+        <v>269</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>368</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>369</v>
+        <v>271</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="19" t="s">
-        <v>370</v>
+        <v>272</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="19" t="s">
-        <v>371</v>
+        <v>273</v>
       </c>
     </row>
   </sheetData>

</xml_diff>